<commit_message>
Complete login test cases and document authentication defects
</commit_message>
<xml_diff>
--- a/docs/TestCases/Test_Cases.xlsx
+++ b/docs/TestCases/Test_Cases.xlsx
@@ -9,7 +9,7 @@
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Tabelle1_2" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="107">
   <si>
     <t xml:space="preserve">Demoblaze Test Cases</t>
   </si>
@@ -443,16 +443,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Leave  username field empty
+      <t xml:space="preserve">  Leave  username field empty
 </t>
     </r>
     <r>
@@ -540,6 +531,698 @@
   </si>
   <si>
     <t xml:space="preserve">Failed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Module 2 : Login/Logout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login with valid credentials </t>
+  </si>
+  <si>
+    <t xml:space="preserve">User is not logged in and on the homepage</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Click Log in
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Enter username
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Enter Password
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Click Log in button</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">User is logged in and landed on home homepage.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attempt login with non-existing credentials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Username : random1199
+Password : random1199</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User receives a „User does not exist.“ pop-up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attempt login with empty username field</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Click Log in
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Leave username field empty
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Enter Password
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Click Log in button</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Log-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attempt login with empty password field</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Click Log in 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Enter username
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Leave Password field empty
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Click Log in button</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Log-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attempt login with valid username and invalid password</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Username : mrdimitrov1234
+Password : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">random1199</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">User receives a generic authentication error message that does not reveal whether the username or password is incorrect.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User receives a „Wrong password.“ pop-up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attempt login with invalid username and valid password</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Username : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">random1199
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Password : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">test1234</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Log-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attempt login with all empty fields</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Click Log in 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">  Leave  username field empty
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Leave Password field empty
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Click Log in button</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Log-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attempt login with only space characters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The application accepts whitespace-only credentials and grants an authenticated session. The navigation bar changes to logged-in state. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login with XSS payload</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Username :  &lt;script&gt;alert('test')&lt;/script&gt; 
+Password :  &lt;script&gt;alert('test')&lt;/script&gt; </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Input should be sanitized.
+Authentication should fail.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The application accepts script-tag input as credentials and grants an authenticated session. The payload is displayed as the logged-in username.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logout by clicking the button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User is logged in</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Click Log out 
+</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">User is logged out and navigated to homepage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User is logged out and landed on homepage for users not logged in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify Logout button is visible after login</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Login with valid credentials </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Observe navigation bar
+</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Logout button is visible after successful login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify Login button is visible after logout</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Click Log out </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Observe navigation bar
+</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Login and Sign up buttons are visible again</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User is logged out and laned on the homepage</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Click Log out 
+</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -549,7 +1232,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -581,12 +1264,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b val="true"/>
       <sz val="16"/>
       <color theme="1"/>
@@ -608,6 +1285,7 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -616,6 +1294,39 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00A933"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFC9211E"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -700,69 +1411,101 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -825,10 +1568,10 @@
       <rgbColor rgb="FF5983B0"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF00A933"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FFC9211E"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
@@ -1017,668 +1760,668 @@
   <dimension ref="A1:W21"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12.36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="35.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="30.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="22.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="21.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="35.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="30.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="22.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="21.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="26.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
-      <c r="W1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2"/>
+      <c r="W1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="4" t="s">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="3" t="s">
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="3"/>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="3"/>
-      <c r="S2" s="3"/>
-      <c r="T2" s="3"/>
-      <c r="U2" s="3"/>
-      <c r="V2" s="3"/>
-      <c r="W2" s="3"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
+      <c r="U2" s="4"/>
+      <c r="V2" s="4"/>
+      <c r="W2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="5" t="s">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="3"/>
-      <c r="P3" s="3"/>
-      <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
-      <c r="S3" s="3"/>
-      <c r="T3" s="3"/>
-      <c r="U3" s="3"/>
-      <c r="V3" s="3"/>
-      <c r="W3" s="3"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+      <c r="S3" s="4"/>
+      <c r="T3" s="4"/>
+      <c r="U3" s="4"/>
+      <c r="V3" s="4"/>
+      <c r="W3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2"/>
-      <c r="B4" s="6" t="s">
+      <c r="A4" s="3"/>
+      <c r="B4" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="U4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
+      <c r="S4" s="4"/>
+      <c r="T4" s="4"/>
+      <c r="U4" s="4"/>
+      <c r="V4" s="4"/>
+      <c r="W4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="7" t="s">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="J5" s="7" t="s">
+      <c r="J5" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="K5" s="7" t="s">
+      <c r="K5" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="L5" s="7" t="s">
+      <c r="L5" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="M5" s="7" t="s">
+      <c r="M5" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="N5" s="7" t="s">
+      <c r="N5" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="O5" s="3"/>
-      <c r="P5" s="3"/>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="3"/>
-      <c r="S5" s="3"/>
-      <c r="T5" s="3"/>
-      <c r="U5" s="3"/>
-      <c r="V5" s="3"/>
-      <c r="W5" s="3"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
+      <c r="U5" s="4"/>
+      <c r="V5" s="4"/>
+      <c r="W5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="9" t="s">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I6" s="11" t="s">
+      <c r="I6" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="10" t="s">
+      <c r="J6" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="K6" s="12" t="s">
+      <c r="K6" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="L6" s="12" t="s">
+      <c r="L6" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="M6" s="10" t="s">
+      <c r="M6" s="11" t="s">
         <v>22</v>
       </c>
       <c r="N6" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="O6" s="3"/>
-      <c r="P6" s="3"/>
-      <c r="Q6" s="3"/>
-      <c r="R6" s="3"/>
-      <c r="S6" s="3"/>
-      <c r="T6" s="3"/>
-      <c r="U6" s="3"/>
-      <c r="V6" s="3"/>
-      <c r="W6" s="3"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
+      <c r="R6" s="4"/>
+      <c r="S6" s="4"/>
+      <c r="T6" s="4"/>
+      <c r="U6" s="4"/>
+      <c r="V6" s="4"/>
+      <c r="W6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="9" t="s">
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I7" s="11" t="s">
+      <c r="I7" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="J7" s="10" t="s">
+      <c r="J7" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="K7" s="10" t="s">
+      <c r="K7" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="L7" s="10" t="s">
+      <c r="L7" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="M7" s="10" t="s">
+      <c r="M7" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="N7" s="10" t="s">
+      <c r="N7" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="O7" s="3"/>
-      <c r="P7" s="3"/>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="3"/>
-      <c r="S7" s="3"/>
-      <c r="T7" s="3"/>
-      <c r="U7" s="3"/>
-      <c r="V7" s="3"/>
-      <c r="W7" s="3"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="4"/>
+      <c r="Q7" s="4"/>
+      <c r="R7" s="4"/>
+      <c r="S7" s="4"/>
+      <c r="T7" s="4"/>
+      <c r="U7" s="4"/>
+      <c r="V7" s="4"/>
+      <c r="W7" s="4"/>
     </row>
     <row r="8" customFormat="false" ht="92.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="9" t="s">
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G8" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I8" s="11" t="s">
+      <c r="I8" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="J8" s="10" t="s">
+      <c r="J8" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="K8" s="10" t="s">
+      <c r="K8" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="L8" s="10" t="s">
+      <c r="L8" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="M8" s="10" t="s">
+      <c r="M8" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="N8" s="10" t="s">
+      <c r="N8" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="O8" s="3"/>
-      <c r="P8" s="3"/>
-      <c r="Q8" s="3"/>
-      <c r="R8" s="3"/>
-      <c r="S8" s="3"/>
-      <c r="T8" s="3"/>
-      <c r="U8" s="3"/>
-      <c r="V8" s="3"/>
-      <c r="W8" s="3"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
+      <c r="R8" s="4"/>
+      <c r="S8" s="4"/>
+      <c r="T8" s="4"/>
+      <c r="U8" s="4"/>
+      <c r="V8" s="4"/>
+      <c r="W8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="92.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="9" t="s">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="G9" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="H9" s="10" t="s">
+      <c r="H9" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I9" s="11" t="s">
+      <c r="I9" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="J9" s="10" t="s">
+      <c r="J9" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="K9" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="L9" s="10" t="s">
+      <c r="L9" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="M9" s="10" t="s">
+      <c r="M9" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="N9" s="10" t="s">
+      <c r="N9" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="O9" s="3"/>
-      <c r="P9" s="3"/>
-      <c r="Q9" s="3"/>
-      <c r="R9" s="3"/>
-      <c r="S9" s="3"/>
-      <c r="T9" s="3"/>
-      <c r="U9" s="3"/>
-      <c r="V9" s="3"/>
-      <c r="W9" s="3"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4"/>
+      <c r="Q9" s="4"/>
+      <c r="R9" s="4"/>
+      <c r="S9" s="4"/>
+      <c r="T9" s="4"/>
+      <c r="U9" s="4"/>
+      <c r="V9" s="4"/>
+      <c r="W9" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="9" t="s">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="G10" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I10" s="11" t="s">
+      <c r="I10" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10" t="s">
+      <c r="J10" s="11"/>
+      <c r="K10" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="L10" s="10" t="s">
+      <c r="L10" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="M10" s="10" t="s">
+      <c r="M10" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="N10" s="10" t="s">
+      <c r="N10" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="O10" s="3"/>
-      <c r="P10" s="3"/>
-      <c r="Q10" s="3"/>
-      <c r="R10" s="3"/>
-      <c r="S10" s="3"/>
-      <c r="T10" s="3"/>
-      <c r="U10" s="3"/>
-      <c r="V10" s="3"/>
-      <c r="W10" s="3"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
+      <c r="Q10" s="4"/>
+      <c r="R10" s="4"/>
+      <c r="S10" s="4"/>
+      <c r="T10" s="4"/>
+      <c r="U10" s="4"/>
+      <c r="V10" s="4"/>
+      <c r="W10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="9" t="s">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="G11" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="H11" s="10" t="s">
+      <c r="H11" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I11" s="11" t="s">
+      <c r="I11" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="J11" s="10" t="s">
+      <c r="J11" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="K11" s="10" t="s">
+      <c r="K11" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="L11" s="12" t="s">
+      <c r="L11" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="M11" s="10" t="s">
+      <c r="M11" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="N11" s="10" t="s">
+      <c r="N11" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="O11" s="3"/>
-      <c r="P11" s="3"/>
-      <c r="Q11" s="3"/>
-      <c r="R11" s="3"/>
-      <c r="S11" s="3"/>
-      <c r="T11" s="3"/>
-      <c r="U11" s="3"/>
-      <c r="V11" s="3"/>
-      <c r="W11" s="3"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="4"/>
+      <c r="Q11" s="4"/>
+      <c r="R11" s="4"/>
+      <c r="S11" s="4"/>
+      <c r="T11" s="4"/>
+      <c r="U11" s="4"/>
+      <c r="V11" s="4"/>
+      <c r="W11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="264.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="9" t="s">
+      <c r="A12" s="4"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="G12" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="H12" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I12" s="11" t="s">
+      <c r="I12" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="J12" s="10" t="s">
+      <c r="J12" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="K12" s="10" t="s">
+      <c r="K12" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="L12" s="12" t="s">
+      <c r="L12" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="M12" s="10" t="s">
+      <c r="M12" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="N12" s="10" t="s">
+      <c r="N12" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="O12" s="3"/>
-      <c r="P12" s="3"/>
-      <c r="Q12" s="3"/>
-      <c r="R12" s="3"/>
-      <c r="S12" s="3"/>
-      <c r="T12" s="3"/>
-      <c r="U12" s="3"/>
-      <c r="V12" s="3"/>
-      <c r="W12" s="3"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="4"/>
+      <c r="Q12" s="4"/>
+      <c r="R12" s="4"/>
+      <c r="S12" s="4"/>
+      <c r="T12" s="4"/>
+      <c r="U12" s="4"/>
+      <c r="V12" s="4"/>
+      <c r="W12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="9" t="s">
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="G13" s="10" t="s">
+      <c r="G13" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="H13" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I13" s="11" t="s">
+      <c r="I13" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="J13" s="10" t="s">
+      <c r="J13" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="K13" s="10" t="s">
+      <c r="K13" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="L13" s="10" t="s">
+      <c r="L13" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="M13" s="10" t="s">
+      <c r="M13" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="N13" s="10" t="s">
+      <c r="N13" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="O13" s="3"/>
-      <c r="P13" s="3"/>
-      <c r="Q13" s="3"/>
-      <c r="R13" s="3"/>
-      <c r="S13" s="3"/>
-      <c r="T13" s="3"/>
-      <c r="U13" s="3"/>
-      <c r="V13" s="3"/>
-      <c r="W13" s="3"/>
+      <c r="O13" s="4"/>
+      <c r="P13" s="4"/>
+      <c r="Q13" s="4"/>
+      <c r="R13" s="4"/>
+      <c r="S13" s="4"/>
+      <c r="T13" s="4"/>
+      <c r="U13" s="4"/>
+      <c r="V13" s="4"/>
+      <c r="W13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="6"/>
-      <c r="M14" s="6"/>
-      <c r="N14" s="6"/>
-      <c r="O14" s="3"/>
-      <c r="P14" s="3"/>
-      <c r="Q14" s="3"/>
-      <c r="R14" s="3"/>
-      <c r="S14" s="3"/>
-      <c r="T14" s="3"/>
-      <c r="U14" s="3"/>
-      <c r="V14" s="3"/>
-      <c r="W14" s="3"/>
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
+      <c r="N14" s="7"/>
+      <c r="O14" s="4"/>
+      <c r="P14" s="4"/>
+      <c r="Q14" s="4"/>
+      <c r="R14" s="4"/>
+      <c r="S14" s="4"/>
+      <c r="T14" s="4"/>
+      <c r="U14" s="4"/>
+      <c r="V14" s="4"/>
+      <c r="W14" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="6"/>
-      <c r="M15" s="6"/>
-      <c r="N15" s="6"/>
-      <c r="O15" s="3"/>
-      <c r="P15" s="3"/>
-      <c r="Q15" s="3"/>
-      <c r="R15" s="3"/>
-      <c r="S15" s="3"/>
-      <c r="T15" s="3"/>
-      <c r="U15" s="3"/>
-      <c r="V15" s="3"/>
-      <c r="W15" s="3"/>
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="7"/>
+      <c r="L15" s="7"/>
+      <c r="M15" s="7"/>
+      <c r="N15" s="7"/>
+      <c r="O15" s="4"/>
+      <c r="P15" s="4"/>
+      <c r="Q15" s="4"/>
+      <c r="R15" s="4"/>
+      <c r="S15" s="4"/>
+      <c r="T15" s="4"/>
+      <c r="U15" s="4"/>
+      <c r="V15" s="4"/>
+      <c r="W15" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="O16" s="3"/>
-      <c r="P16" s="3"/>
-      <c r="Q16" s="3"/>
-      <c r="R16" s="3"/>
-      <c r="S16" s="3"/>
-      <c r="T16" s="3"/>
-      <c r="U16" s="3"/>
-      <c r="V16" s="3"/>
-      <c r="W16" s="3"/>
+      <c r="A16" s="4"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="O16" s="4"/>
+      <c r="P16" s="4"/>
+      <c r="Q16" s="4"/>
+      <c r="R16" s="4"/>
+      <c r="S16" s="4"/>
+      <c r="T16" s="4"/>
+      <c r="U16" s="4"/>
+      <c r="V16" s="4"/>
+      <c r="W16" s="4"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="O17" s="3"/>
-      <c r="P17" s="3"/>
-      <c r="Q17" s="3"/>
-      <c r="R17" s="3"/>
-      <c r="S17" s="3"/>
-      <c r="T17" s="3"/>
-      <c r="U17" s="3"/>
-      <c r="V17" s="3"/>
-      <c r="W17" s="3"/>
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="O17" s="4"/>
+      <c r="P17" s="4"/>
+      <c r="Q17" s="4"/>
+      <c r="R17" s="4"/>
+      <c r="S17" s="4"/>
+      <c r="T17" s="4"/>
+      <c r="U17" s="4"/>
+      <c r="V17" s="4"/>
+      <c r="W17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="O18" s="3"/>
-      <c r="P18" s="3"/>
-      <c r="Q18" s="3"/>
-      <c r="R18" s="3"/>
-      <c r="S18" s="3"/>
-      <c r="T18" s="3"/>
-      <c r="U18" s="3"/>
-      <c r="V18" s="3"/>
-      <c r="W18" s="3"/>
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="O18" s="4"/>
+      <c r="P18" s="4"/>
+      <c r="Q18" s="4"/>
+      <c r="R18" s="4"/>
+      <c r="S18" s="4"/>
+      <c r="T18" s="4"/>
+      <c r="U18" s="4"/>
+      <c r="V18" s="4"/>
+      <c r="W18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="42.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="O19" s="3"/>
-      <c r="P19" s="3"/>
-      <c r="Q19" s="3"/>
-      <c r="R19" s="3"/>
-      <c r="S19" s="3"/>
-      <c r="T19" s="3"/>
-      <c r="U19" s="3"/>
-      <c r="V19" s="3"/>
-      <c r="W19" s="3"/>
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="O19" s="4"/>
+      <c r="P19" s="4"/>
+      <c r="Q19" s="4"/>
+      <c r="R19" s="4"/>
+      <c r="S19" s="4"/>
+      <c r="T19" s="4"/>
+      <c r="U19" s="4"/>
+      <c r="V19" s="4"/>
+      <c r="W19" s="4"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="O20" s="3"/>
-      <c r="P20" s="3"/>
-      <c r="Q20" s="3"/>
-      <c r="R20" s="3"/>
-      <c r="S20" s="3"/>
-      <c r="T20" s="3"/>
-      <c r="U20" s="3"/>
-      <c r="V20" s="3"/>
-      <c r="W20" s="3"/>
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="O20" s="4"/>
+      <c r="P20" s="4"/>
+      <c r="Q20" s="4"/>
+      <c r="R20" s="4"/>
+      <c r="S20" s="4"/>
+      <c r="T20" s="4"/>
+      <c r="U20" s="4"/>
+      <c r="V20" s="4"/>
+      <c r="W20" s="4"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="O21" s="3"/>
-      <c r="P21" s="3"/>
-      <c r="Q21" s="3"/>
-      <c r="R21" s="3"/>
-      <c r="S21" s="3"/>
-      <c r="T21" s="3"/>
-      <c r="U21" s="3"/>
-      <c r="V21" s="3"/>
-      <c r="W21" s="3"/>
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="O21" s="4"/>
+      <c r="P21" s="4"/>
+      <c r="Q21" s="4"/>
+      <c r="R21" s="4"/>
+      <c r="S21" s="4"/>
+      <c r="T21" s="4"/>
+      <c r="U21" s="4"/>
+      <c r="V21" s="4"/>
+      <c r="W21" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1714,89 +2457,876 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:W25"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15.32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="20.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="17.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="27.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="19.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="16.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="14.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="23.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="35.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="30.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="22.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="21.14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O1" s="3"/>
-    </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O2" s="3"/>
-    </row>
-    <row r="3" customFormat="false" ht="150.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="O3" s="3"/>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O4" s="3"/>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O5" s="3"/>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O6" s="3"/>
-    </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O7" s="3"/>
-    </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O8" s="3"/>
-    </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O9" s="3"/>
-    </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O10" s="3"/>
-    </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O11" s="3"/>
-    </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O12" s="3"/>
-    </row>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-      <c r="O13" s="3"/>
-    </row>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D14" s="3"/>
-    </row>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D15" s="3"/>
-    </row>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D16" s="3"/>
+    <row r="1" customFormat="false" ht="26.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2"/>
+      <c r="W1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
+      <c r="U2" s="4"/>
+      <c r="V2" s="4"/>
+      <c r="W2" s="4"/>
+    </row>
+    <row r="3" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+      <c r="S3" s="4"/>
+      <c r="T3" s="4"/>
+      <c r="U3" s="4"/>
+      <c r="V3" s="4"/>
+      <c r="W3" s="4"/>
+    </row>
+    <row r="4" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3"/>
+      <c r="B4" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
+      <c r="S4" s="4"/>
+      <c r="T4" s="4"/>
+      <c r="U4" s="4"/>
+      <c r="V4" s="4"/>
+      <c r="W4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="L5" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="M5" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="N5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
+      <c r="U5" s="4"/>
+      <c r="V5" s="4"/>
+      <c r="W5" s="4"/>
+    </row>
+    <row r="6" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="I6" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="L6" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="M6" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="N6" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
+      <c r="R6" s="4"/>
+      <c r="S6" s="4"/>
+      <c r="T6" s="4"/>
+      <c r="U6" s="4"/>
+      <c r="V6" s="4"/>
+      <c r="W6" s="4"/>
+    </row>
+    <row r="7" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="I7" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="L7" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="M7" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="N7" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="O7" s="4"/>
+      <c r="P7" s="4"/>
+      <c r="Q7" s="4"/>
+      <c r="R7" s="4"/>
+      <c r="S7" s="4"/>
+      <c r="T7" s="4"/>
+      <c r="U7" s="4"/>
+      <c r="V7" s="4"/>
+      <c r="W7" s="4"/>
+    </row>
+    <row r="8" customFormat="false" ht="92.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="I8" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="J8" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="L8" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="M8" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="N8" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
+      <c r="R8" s="4"/>
+      <c r="S8" s="4"/>
+      <c r="T8" s="4"/>
+      <c r="U8" s="4"/>
+      <c r="V8" s="4"/>
+      <c r="W8" s="4"/>
+    </row>
+    <row r="9" customFormat="false" ht="92.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="I9" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="J9" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="L9" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="M9" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="N9" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4"/>
+      <c r="Q9" s="4"/>
+      <c r="R9" s="4"/>
+      <c r="S9" s="4"/>
+      <c r="T9" s="4"/>
+      <c r="U9" s="4"/>
+      <c r="V9" s="4"/>
+      <c r="W9" s="4"/>
+    </row>
+    <row r="10" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="H10" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="I10" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="J10" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="K10" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="L10" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="M10" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="N10" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
+      <c r="Q10" s="4"/>
+      <c r="R10" s="4"/>
+      <c r="S10" s="4"/>
+      <c r="T10" s="4"/>
+      <c r="U10" s="4"/>
+      <c r="V10" s="4"/>
+      <c r="W10" s="4"/>
+    </row>
+    <row r="11" customFormat="false" ht="81.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="H11" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="I11" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="J11" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="K11" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="L11" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="M11" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="N11" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="O11" s="4"/>
+      <c r="P11" s="4"/>
+      <c r="Q11" s="4"/>
+      <c r="R11" s="4"/>
+      <c r="S11" s="4"/>
+      <c r="T11" s="4"/>
+      <c r="U11" s="4"/>
+      <c r="V11" s="4"/>
+      <c r="W11" s="4"/>
+    </row>
+    <row r="12" customFormat="false" ht="104.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="I12" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="J12" s="11"/>
+      <c r="K12" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="L12" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="M12" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="N12" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="O12" s="4"/>
+      <c r="P12" s="4"/>
+      <c r="Q12" s="4"/>
+      <c r="R12" s="4"/>
+      <c r="S12" s="4"/>
+      <c r="T12" s="4"/>
+      <c r="U12" s="4"/>
+      <c r="V12" s="4"/>
+      <c r="W12" s="4"/>
+    </row>
+    <row r="13" customFormat="false" ht="80.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="H13" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="I13" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="J13" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="K13" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="L13" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="M13" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="N13" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="O13" s="4"/>
+      <c r="P13" s="4"/>
+      <c r="Q13" s="4"/>
+      <c r="R13" s="4"/>
+      <c r="S13" s="4"/>
+      <c r="T13" s="4"/>
+      <c r="U13" s="4"/>
+      <c r="V13" s="4"/>
+      <c r="W13" s="4"/>
+    </row>
+    <row r="14" customFormat="false" ht="89.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="H14" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="I14" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="J14" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="K14" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="L14" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="M14" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="N14" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="O14" s="4"/>
+      <c r="P14" s="4"/>
+      <c r="Q14" s="4"/>
+      <c r="R14" s="4"/>
+      <c r="S14" s="4"/>
+      <c r="T14" s="4"/>
+      <c r="U14" s="4"/>
+      <c r="V14" s="4"/>
+      <c r="W14" s="4"/>
+    </row>
+    <row r="15" customFormat="false" ht="51.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="H15" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="I15" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="J15" s="11"/>
+      <c r="K15" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="L15" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="M15" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="N15" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="O15" s="4"/>
+      <c r="P15" s="4"/>
+      <c r="Q15" s="4"/>
+      <c r="R15" s="4"/>
+      <c r="S15" s="4"/>
+      <c r="T15" s="4"/>
+      <c r="U15" s="4"/>
+      <c r="V15" s="4"/>
+      <c r="W15" s="4"/>
+    </row>
+    <row r="16" customFormat="false" ht="78.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="G16" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="H16" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="I16" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="J16" s="11"/>
+      <c r="K16" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="L16" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="M16" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="N16" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="O16" s="4"/>
+      <c r="P16" s="4"/>
+      <c r="Q16" s="4"/>
+      <c r="R16" s="4"/>
+      <c r="S16" s="4"/>
+      <c r="T16" s="4"/>
+      <c r="U16" s="4"/>
+      <c r="V16" s="4"/>
+      <c r="W16" s="4"/>
+    </row>
+    <row r="17" customFormat="false" ht="60.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="H17" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="I17" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="L17" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="M17" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="N17" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="O17" s="4"/>
+      <c r="P17" s="4"/>
+      <c r="Q17" s="4"/>
+      <c r="R17" s="4"/>
+      <c r="S17" s="4"/>
+      <c r="T17" s="4"/>
+      <c r="U17" s="4"/>
+      <c r="V17" s="4"/>
+      <c r="W17" s="4"/>
+    </row>
+    <row r="18" customFormat="false" ht="65.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="I18" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="J18" s="11"/>
+      <c r="K18" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="L18" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="M18" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="N18" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="O18" s="4"/>
+      <c r="P18" s="4"/>
+      <c r="Q18" s="4"/>
+      <c r="R18" s="4"/>
+      <c r="S18" s="4"/>
+      <c r="T18" s="4"/>
+      <c r="U18" s="4"/>
+      <c r="V18" s="4"/>
+      <c r="W18" s="4"/>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="J19" s="23"/>
+      <c r="O19" s="4"/>
+      <c r="P19" s="4"/>
+      <c r="Q19" s="4"/>
+      <c r="R19" s="4"/>
+      <c r="S19" s="4"/>
+      <c r="T19" s="4"/>
+      <c r="U19" s="4"/>
+      <c r="V19" s="4"/>
+      <c r="W19" s="4"/>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="O20" s="4"/>
+      <c r="P20" s="4"/>
+      <c r="Q20" s="4"/>
+      <c r="R20" s="4"/>
+      <c r="S20" s="4"/>
+      <c r="T20" s="4"/>
+      <c r="U20" s="4"/>
+      <c r="V20" s="4"/>
+      <c r="W20" s="4"/>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="O21" s="4"/>
+      <c r="P21" s="4"/>
+      <c r="Q21" s="4"/>
+      <c r="R21" s="4"/>
+      <c r="S21" s="4"/>
+      <c r="T21" s="4"/>
+      <c r="U21" s="4"/>
+      <c r="V21" s="4"/>
+      <c r="W21" s="4"/>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="O22" s="4"/>
+      <c r="P22" s="4"/>
+      <c r="Q22" s="4"/>
+      <c r="R22" s="4"/>
+      <c r="S22" s="4"/>
+      <c r="T22" s="4"/>
+      <c r="U22" s="4"/>
+      <c r="V22" s="4"/>
+      <c r="W22" s="4"/>
+    </row>
+    <row r="23" customFormat="false" ht="42.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="O23" s="4"/>
+      <c r="P23" s="4"/>
+      <c r="Q23" s="4"/>
+      <c r="R23" s="4"/>
+      <c r="S23" s="4"/>
+      <c r="T23" s="4"/>
+      <c r="U23" s="4"/>
+      <c r="V23" s="4"/>
+      <c r="W23" s="4"/>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="O24" s="4"/>
+      <c r="P24" s="4"/>
+      <c r="Q24" s="4"/>
+      <c r="R24" s="4"/>
+      <c r="S24" s="4"/>
+      <c r="T24" s="4"/>
+      <c r="U24" s="4"/>
+      <c r="V24" s="4"/>
+      <c r="W24" s="4"/>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="O25" s="4"/>
+      <c r="P25" s="4"/>
+      <c r="Q25" s="4"/>
+      <c r="R25" s="4"/>
+      <c r="S25" s="4"/>
+      <c r="T25" s="4"/>
+      <c r="U25" s="4"/>
+      <c r="V25" s="4"/>
+      <c r="W25" s="4"/>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:W1"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="E3:N3"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="M6:M18" type="list">
+      <formula1>"High,Medium,Low"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="N6:N18" type="list">
+      <formula1>"Not Run,Passed,Failed,Blocked"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="H2" r:id="rId1" display=" https://www.demoblaze.com/"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader/>
+    <oddFooter/>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>